<commit_message>
Update: Added method in util for Autosuggestion and also configure some method to propertis file
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
@@ -73,30 +73,6 @@
     <t>expDataId</t>
   </si>
   <si>
-    <t>ID-1</t>
-  </si>
-  <si>
-    <t>ID-2</t>
-  </si>
-  <si>
-    <t>ID-3</t>
-  </si>
-  <si>
-    <t>ID-4</t>
-  </si>
-  <si>
-    <t>ID-5</t>
-  </si>
-  <si>
-    <t>ID-6</t>
-  </si>
-  <si>
-    <t>ID-7</t>
-  </si>
-  <si>
-    <t>ID-8</t>
-  </si>
-  <si>
     <t>type</t>
   </si>
   <si>
@@ -164,6 +140,30 @@
   </si>
   <si>
     <t>valid</t>
+  </si>
+  <si>
+    <t>M-1</t>
+  </si>
+  <si>
+    <t>M-2</t>
+  </si>
+  <si>
+    <t>M-3</t>
+  </si>
+  <si>
+    <t>M-4</t>
+  </si>
+  <si>
+    <t>A-1</t>
+  </si>
+  <si>
+    <t>A-2</t>
+  </si>
+  <si>
+    <t>A-3</t>
+  </si>
+  <si>
+    <t>A-4</t>
   </si>
 </sst>
 </file>
@@ -511,7 +511,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -534,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -548,10 +548,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -562,10 +562,10 @@
         <v>123</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -576,10 +576,10 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -616,16 +616,16 @@
         <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -639,16 +639,16 @@
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -662,16 +662,16 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -685,16 +685,16 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -708,16 +708,16 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -731,16 +731,16 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
         <v>32</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -754,16 +754,16 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" t="s">
         <v>33</v>
-      </c>
-      <c r="G7" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -777,16 +777,16 @@
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -800,16 +800,16 @@
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -847,7 +847,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -861,7 +861,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -875,7 +875,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -903,7 +903,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -917,7 +917,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -931,7 +931,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
@@ -972,18 +972,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactored naming conventions and added POJO package and classes for test case management
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="121">
   <si>
     <t>username</t>
   </si>
@@ -376,6 +376,9 @@
   </si>
   <si>
     <t>Master Party Duplicate Government Shipper IEC</t>
+  </si>
+  <si>
+    <t>7543210123</t>
   </si>
 </sst>
 </file>
@@ -731,7 +734,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1409,7 +1412,7 @@
         <v>117</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
Added new testcases for deltion in Masters
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="123">
   <si>
     <t>username</t>
   </si>
@@ -333,9 +333,6 @@
     <t>ShipperPartySearch</t>
   </si>
   <si>
-    <t>ShipperPartyDeletion</t>
-  </si>
-  <si>
     <t>14</t>
   </si>
   <si>
@@ -379,6 +376,15 @@
   </si>
   <si>
     <t>7543210123</t>
+  </si>
+  <si>
+    <t>GovernmentShipperPartyDeletion</t>
+  </si>
+  <si>
+    <t>PrivateShipperPartyDeletion</t>
+  </si>
+  <si>
+    <t>DuplicateGovernmentShipperPartyDeletion</t>
   </si>
 </sst>
 </file>
@@ -734,7 +740,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1165,7 +1171,7 @@
         <v>101</v>
       </c>
       <c r="E2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>91</v>
@@ -1212,7 +1218,7 @@
         <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>92</v>
@@ -1259,7 +1265,7 @@
         <v>102</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>92</v>
@@ -1271,10 +1277,10 @@
         <v>67</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K4" t="s">
         <v>53</v>
@@ -1295,7 +1301,7 @@
         <v>97</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="R4" t="s">
         <v>79</v>
@@ -1306,7 +1312,7 @@
         <v>90</v>
       </c>
       <c r="E5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>92</v>
@@ -1318,10 +1324,10 @@
         <v>69</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K5" t="s">
         <v>53</v>
@@ -1342,7 +1348,7 @@
         <v>73</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="R5" t="s">
         <v>51</v>
@@ -1353,7 +1359,7 @@
         <v>95</v>
       </c>
       <c r="E6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>91</v>
@@ -1365,7 +1371,7 @@
         <v>67</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>78</v>
@@ -1389,7 +1395,7 @@
         <v>47</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R6" t="s">
         <v>96</v>
@@ -1406,13 +1412,13 @@
         <v>88</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>66</v>
@@ -1445,7 +1451,7 @@
         <v>73</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R7" t="s">
         <v>84</v>
@@ -1462,7 +1468,7 @@
         <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
@@ -1472,7 +1478,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="B9" t="s">
         <v>66</v>
@@ -1481,7 +1487,7 @@
         <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
@@ -1493,18 +1499,48 @@
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" t="s">
+        <v>118</v>
+      </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="Q10" s="7"/>
+      <c r="R10" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" t="s">
+        <v>115</v>
+      </c>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="Q11" s="7"/>
+      <c r="R11" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F12" s="7"/>

</xml_diff>

<commit_message>
Configure jenkin server open automatically
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -4,19 +4,20 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
     <sheet name="All_BranchSheet" sheetId="3" r:id="rId2"/>
     <sheet name="MastersPartyExporter" sheetId="5" r:id="rId3"/>
+    <sheet name="MastersPartyConsignee" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="124">
   <si>
     <t>username</t>
   </si>
@@ -385,6 +386,9 @@
   </si>
   <si>
     <t>DuplicateGovernmentShipperPartyDeletion</t>
+  </si>
+  <si>
+    <t>ConsigneePartyCreation</t>
   </si>
 </sst>
 </file>
@@ -1553,4 +1557,92 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Configure Email from jenkins for pass & fail result
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="132">
   <si>
     <t>username</t>
   </si>
@@ -389,13 +389,37 @@
   </si>
   <si>
     <t>ConsigneePartyCreation</t>
+  </si>
+  <si>
+    <t>selectRadioButton</t>
+  </si>
+  <si>
+    <t>rdoConsignee</t>
+  </si>
+  <si>
+    <t>Master Consignee Creation</t>
+  </si>
+  <si>
+    <t>extendedName</t>
+  </si>
+  <si>
+    <t>Consignee/Supplier</t>
+  </si>
+  <si>
+    <t>New Delhi 12/22</t>
+  </si>
+  <si>
+    <t>contactPerson</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -434,6 +458,17 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6A3E3E"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -456,7 +491,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -471,6 +506,8 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -744,7 +781,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1561,27 +1598,28 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>81</v>
       </c>
@@ -1594,55 +1632,67 @@
       <c r="D1" t="s">
         <v>89</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="G1" s="6" t="s">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>130</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="M1" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N1" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>123</v>
       </c>
+      <c r="E2" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="F2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H2" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" t="s">
+        <v>131</v>
+      </c>
+      <c r="J2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" t="s">
+        <v>47</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chnages in jenkins file for getiing pass failed report properly in email
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="135">
   <si>
     <t>username</t>
   </si>
@@ -413,6 +413,15 @@
   </si>
   <si>
     <t>Test</t>
+  </si>
+  <si>
+    <t>verifyShipperPartyEnteredDetailsAreClear</t>
+  </si>
+  <si>
+    <t>TC_04</t>
+  </si>
+  <si>
+    <t>User Already Login.</t>
   </si>
 </sst>
 </file>
@@ -781,7 +790,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -789,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
@@ -865,12 +874,30 @@
         <v>61</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1"/>
+    <hyperlink ref="C5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1131,7 +1158,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41" bestFit="1" customWidth="1"/>
@@ -1519,29 +1546,51 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>120</v>
-      </c>
-      <c r="B9" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" t="s">
-        <v>116</v>
-      </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" t="s">
-        <v>85</v>
+      <c r="H9" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="K9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L9" t="s">
+        <v>48</v>
+      </c>
+      <c r="M9" t="s">
+        <v>98</v>
+      </c>
+      <c r="N9" t="s">
+        <v>97</v>
+      </c>
+      <c r="O9" t="s">
+        <v>99</v>
+      </c>
+      <c r="P9" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B10" t="s">
         <v>66</v>
@@ -1550,7 +1599,7 @@
         <v>88</v>
       </c>
       <c r="D10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
@@ -1563,16 +1612,16 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
         <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
@@ -1584,11 +1633,33 @@
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" t="s">
+        <v>115</v>
+      </c>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="Q12" s="7"/>
+      <c r="R12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="Q13" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rechange ij jenkins file
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="133">
   <si>
     <t>username</t>
   </si>
@@ -416,12 +416,6 @@
   </si>
   <si>
     <t>verifyShipperPartyEnteredDetailsAreClear</t>
-  </si>
-  <si>
-    <t>TC_04</t>
-  </si>
-  <si>
-    <t>User Already Login.</t>
   </si>
 </sst>
 </file>
@@ -790,7 +784,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -875,29 +869,16 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>134</v>
-      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2"/>
+      <c r="E5" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1"/>
-    <hyperlink ref="C5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
check if failed test case disaplyed in email and jenkins
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="134">
   <si>
     <t>username</t>
   </si>
@@ -416,6 +416,9 @@
   </si>
   <si>
     <t>verifyShipperPartyEnteredDetailsAreClear</t>
+  </si>
+  <si>
+    <t>iCaffe..</t>
   </si>
 </sst>
 </file>
@@ -784,7 +787,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -792,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
@@ -828,7 +831,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>62</v>
@@ -867,11 +870,6 @@
       <c r="E4" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="1"/>
-      <c r="C5" s="2"/>
-      <c r="E5" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Re changes in validation code for login for checking failed email testcase
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="133">
   <si>
     <t>username</t>
   </si>
@@ -416,9 +416,6 @@
   </si>
   <si>
     <t>verifyShipperPartyEnteredDetailsAreClear</t>
-  </si>
-  <si>
-    <t>iCaffe..</t>
   </si>
 </sst>
 </file>
@@ -831,7 +828,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
Changes in Jenkins file
</commit_message>
<xml_diff>
--- a/src/test/resources/Akash_TestByDataprovider.xlsx
+++ b/src/test/resources/Akash_TestByDataprovider.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15600" windowHeight="7860" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LoginSheet" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="172">
   <si>
     <t>username</t>
   </si>
@@ -388,34 +388,151 @@
     <t>DuplicateGovernmentShipperPartyDeletion</t>
   </si>
   <si>
-    <t>ConsigneePartyCreation</t>
-  </si>
-  <si>
-    <t>selectRadioButton</t>
-  </si>
-  <si>
     <t>rdoConsignee</t>
   </si>
   <si>
-    <t>Master Consignee Creation</t>
-  </si>
-  <si>
-    <t>extendedName</t>
-  </si>
-  <si>
-    <t>Consignee/Supplier</t>
-  </si>
-  <si>
     <t>New Delhi 12/22</t>
   </si>
   <si>
-    <t>contactPerson</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
     <t>verifyShipperPartyEnteredDetailsAreClear</t>
+  </si>
+  <si>
+    <t>ConsigneeSupplierPartyCreation</t>
+  </si>
+  <si>
+    <t>selectConsigneeType_InSearch</t>
+  </si>
+  <si>
+    <t>selectPartyName_InSearchGrid</t>
+  </si>
+  <si>
+    <t>selSubTypeRaidioBT</t>
+  </si>
+  <si>
+    <t>Supplier Consignee Creation</t>
+  </si>
+  <si>
+    <t>for Master</t>
+  </si>
+  <si>
+    <t>entEmail</t>
+  </si>
+  <si>
+    <t>Supplier@gmail.com</t>
+  </si>
+  <si>
+    <t>Consignee Saved successfully</t>
+  </si>
+  <si>
+    <t>entContactPerson</t>
+  </si>
+  <si>
+    <t>entExtendedName</t>
+  </si>
+  <si>
+    <t>ConsigneeBuyerPartyCreation</t>
+  </si>
+  <si>
+    <t>Buyer Consignee Creation</t>
+  </si>
+  <si>
+    <t>Supplier Test</t>
+  </si>
+  <si>
+    <t>Buyer Test</t>
+  </si>
+  <si>
+    <t>Buyer@gmail.com</t>
+  </si>
+  <si>
+    <t>rdoBuyer</t>
+  </si>
+  <si>
+    <t>ConsigneeNotifyPartyCreation</t>
+  </si>
+  <si>
+    <t>rdoNotify</t>
+  </si>
+  <si>
+    <t>Notify Consignee Creation</t>
+  </si>
+  <si>
+    <t>Mumbai  22/23</t>
+  </si>
+  <si>
+    <t>Gujrat  33/24</t>
+  </si>
+  <si>
+    <t>Notify Test</t>
+  </si>
+  <si>
+    <t>Gujrat</t>
+  </si>
+  <si>
+    <t>Notify</t>
+  </si>
+  <si>
+    <t>Notify@gmail.com</t>
+  </si>
+  <si>
+    <t>CreateShipperPartyWithoutMandatoryFields</t>
+  </si>
+  <si>
+    <t>Please Enter Shipper Name</t>
+  </si>
+  <si>
+    <t>ConsigneeSupplierPartyModification</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>Supplier Consignee Modification</t>
+  </si>
+  <si>
+    <t>for Master Test</t>
+  </si>
+  <si>
+    <t>UttarPradesh</t>
+  </si>
+  <si>
+    <t>UttarPradesh 105/7</t>
+  </si>
+  <si>
+    <t>SupplierTest@gmail.com</t>
+  </si>
+  <si>
+    <t>Consignee Modify successfully</t>
+  </si>
+  <si>
+    <t>Buyer Consignee Modification</t>
+  </si>
+  <si>
+    <t>Lucknow 10/7</t>
+  </si>
+  <si>
+    <t>BuyerTest@gmail.com</t>
+  </si>
+  <si>
+    <t>ConsigneeBuyerPartyModification</t>
+  </si>
+  <si>
+    <t>Buyer</t>
+  </si>
+  <si>
+    <t>ConsigneeNotifyPartyModification</t>
+  </si>
+  <si>
+    <t>Notify Consignee Modification</t>
+  </si>
+  <si>
+    <t>Bhwali 15/7</t>
+  </si>
+  <si>
+    <t>Uttrakhand</t>
+  </si>
+  <si>
+    <t>NotifyTest@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -494,7 +611,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -510,7 +627,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1522,7 +1645,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E9" t="s">
         <v>114</v>
@@ -1631,11 +1754,17 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>152</v>
+      </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
       <c r="Q13" s="7"/>
+      <c r="R13" t="s">
+        <v>153</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1645,101 +1774,273 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D1" t="s">
-        <v>89</v>
-      </c>
-      <c r="E1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F1" s="6" t="s">
+      <c r="B1" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="H1" s="6" t="s">
+      <c r="F1" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="G1" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="J1" s="6" t="s">
+      <c r="H1" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="I1" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="J1" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="K1" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="M1" s="6"/>
+      <c r="L1" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>59</v>
+      </c>
       <c r="N1" s="6"/>
       <c r="O1" s="6"/>
       <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="F2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>128</v>
+      <c r="E2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G2" t="s">
+        <v>124</v>
       </c>
       <c r="H2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="I2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="M2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="J2" t="s">
+      <c r="G3" t="s">
+        <v>146</v>
+      </c>
+      <c r="H3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I3" t="s">
         <v>53</v>
       </c>
-      <c r="K2" t="s">
+      <c r="J3" t="s">
         <v>48</v>
       </c>
-      <c r="L2" t="s">
-        <v>47</v>
+      <c r="K3" t="s">
+        <v>73</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="M3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G4" t="s">
+        <v>147</v>
+      </c>
+      <c r="H4" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" t="s">
+        <v>149</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="M4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="G5" t="s">
+        <v>159</v>
+      </c>
+      <c r="K5" t="s">
+        <v>158</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="M5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="G6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K6" t="s">
+        <v>158</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="M6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B7" t="s">
+        <v>150</v>
+      </c>
+      <c r="C7" t="s">
+        <v>145</v>
+      </c>
+      <c r="E7" t="s">
+        <v>168</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="G7" t="s">
+        <v>169</v>
+      </c>
+      <c r="K7" t="s">
+        <v>170</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="M7" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L2" r:id="rId1"/>
+    <hyperlink ref="L3" r:id="rId2"/>
+    <hyperlink ref="L4" r:id="rId3"/>
+    <hyperlink ref="L5" r:id="rId4"/>
+    <hyperlink ref="L6" r:id="rId5"/>
+    <hyperlink ref="L7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>